<commit_message>
WealthScale: 007 and 008 published October 27
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016xNLX8NWZ1yQW1gWXDEVVM
</commit_message>
<xml_diff>
--- a/wealthscale/WealthScale_201_Pages_Index.xlsx
+++ b/wealthscale/WealthScale_201_Pages_Index.xlsx
@@ -15885,7 +15885,7 @@
       </c>
       <c r="M101" s="10" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done Oct 27 (published before written legal approval; draft note removed)</t>
         </is>
       </c>
     </row>
@@ -15948,7 +15948,7 @@
       </c>
       <c r="M102" s="10" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done Oct 27 (published before written legal approval; draft note removed)</t>
         </is>
       </c>
     </row>
@@ -16007,7 +16007,7 @@
           <t>Why</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -16037,7 +16037,7 @@
           <t>The old page is no longer part of the site plan; this page takes its place</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Done Oct 27: published, 301 added, old page in Trash</t>
         </is>
@@ -16067,7 +16067,7 @@
           <t>The old page is no longer part of the site plan; this page takes its place</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>Done Oct 27: published, 301 added, old page in Trash</t>
         </is>
@@ -16097,7 +16097,7 @@
           <t>The old page is no longer part of the site plan; this page takes its place</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Done Oct 27: published, 301 added, old page in Trash</t>
         </is>

</xml_diff>

<commit_message>
WealthScale re-do day 2: October 28 rows marked Done, workbook recalculated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016xNLX8NWZ1yQW1gWXDEVVM
</commit_message>
<xml_diff>
--- a/wealthscale/WealthScale_201_Pages_Index.xlsx
+++ b/wealthscale/WealthScale_201_Pages_Index.xlsx
@@ -12060,11 +12060,11 @@
       </c>
       <c r="E3" s="3" t="n">
         <f aca="false">COUNTIFS('First 101 pages (latest)'!A$2:A$102,B3,'First 101 pages (latest)'!M$2:M$102,"Done")</f>
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="F3" s="3" t="n">
         <f aca="false">D3-E3</f>
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="G3" s="5" t="n">
         <f aca="false">SUMIF('First 101 pages (latest)'!A$2:A$102,B3,'First 101 pages (latest)'!L$2:L$102)</f>
@@ -12241,11 +12241,11 @@
       </c>
       <c r="E10" s="3" t="n">
         <f aca="false">SUM(E2:E9)</f>
-        <v>52</v>
+        <v>101</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F2:F9)</f>
-        <v>149</v>
+        <v>100</v>
       </c>
       <c r="G10" s="5" t="n">
         <f aca="false">SUM(G2:G9)</f>
@@ -14415,7 +14415,7 @@
         <v>7303</v>
       </c>
       <c r="M52" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14456,7 +14456,7 @@
         <v>7316</v>
       </c>
       <c r="M53" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14497,7 +14497,7 @@
         <v>13645</v>
       </c>
       <c r="M54" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14538,7 +14538,7 @@
         <v>9472</v>
       </c>
       <c r="M55" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14579,7 +14579,7 @@
         <v>11122</v>
       </c>
       <c r="M56" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14620,7 +14620,7 @@
         <v>11797</v>
       </c>
       <c r="M57" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14661,7 +14661,7 @@
         <v>11185</v>
       </c>
       <c r="M58" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14702,7 +14702,7 @@
         <v>9526</v>
       </c>
       <c r="M59" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14743,7 +14743,7 @@
         <v>10260</v>
       </c>
       <c r="M60" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14784,7 +14784,7 @@
         <v>11548</v>
       </c>
       <c r="M61" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14825,7 +14825,7 @@
         <v>9775</v>
       </c>
       <c r="M62" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14866,7 +14866,7 @@
         <v>10327</v>
       </c>
       <c r="M63" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14907,7 +14907,7 @@
         <v>11007</v>
       </c>
       <c r="M64" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14948,7 +14948,7 @@
         <v>11987</v>
       </c>
       <c r="M65" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14989,7 +14989,7 @@
         <v>9991</v>
       </c>
       <c r="M66" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15030,7 +15030,7 @@
         <v>8952</v>
       </c>
       <c r="M67" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15071,7 +15071,7 @@
         <v>10575</v>
       </c>
       <c r="M68" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15112,7 +15112,7 @@
         <v>10855</v>
       </c>
       <c r="M69" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15153,7 +15153,7 @@
         <v>8651</v>
       </c>
       <c r="M70" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15194,7 +15194,7 @@
         <v>9010</v>
       </c>
       <c r="M71" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15235,7 +15235,7 @@
         <v>7961</v>
       </c>
       <c r="M72" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15276,7 +15276,7 @@
         <v>12011</v>
       </c>
       <c r="M73" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15317,7 +15317,7 @@
         <v>8177</v>
       </c>
       <c r="M74" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15358,7 +15358,7 @@
         <v>9158</v>
       </c>
       <c r="M75" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15399,7 +15399,7 @@
         <v>6938</v>
       </c>
       <c r="M76" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15440,7 +15440,7 @@
         <v>7734</v>
       </c>
       <c r="M77" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15481,7 +15481,7 @@
         <v>7602</v>
       </c>
       <c r="M78" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15522,7 +15522,7 @@
         <v>7450</v>
       </c>
       <c r="M79" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15563,7 +15563,7 @@
         <v>6987</v>
       </c>
       <c r="M80" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15604,7 +15604,7 @@
         <v>7114</v>
       </c>
       <c r="M81" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15645,7 +15645,7 @@
         <v>8655</v>
       </c>
       <c r="M82" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15686,7 +15686,7 @@
         <v>8239</v>
       </c>
       <c r="M83" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15727,7 +15727,7 @@
         <v>8021</v>
       </c>
       <c r="M84" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15768,7 +15768,7 @@
         <v>7480</v>
       </c>
       <c r="M85" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15809,7 +15809,7 @@
         <v>7087</v>
       </c>
       <c r="M86" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15850,7 +15850,7 @@
         <v>6846</v>
       </c>
       <c r="M87" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15891,7 +15891,7 @@
         <v>6106</v>
       </c>
       <c r="M88" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15932,7 +15932,7 @@
         <v>5490</v>
       </c>
       <c r="M89" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15973,7 +15973,7 @@
         <v>6535</v>
       </c>
       <c r="M90" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16014,7 +16014,7 @@
         <v>6366</v>
       </c>
       <c r="M91" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16055,7 +16055,7 @@
         <v>6623</v>
       </c>
       <c r="M92" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16096,7 +16096,7 @@
         <v>6429</v>
       </c>
       <c r="M93" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16137,7 +16137,7 @@
         <v>6712</v>
       </c>
       <c r="M94" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16178,7 +16178,7 @@
         <v>6524</v>
       </c>
       <c r="M95" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16219,7 +16219,7 @@
         <v>7611</v>
       </c>
       <c r="M96" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16260,7 +16260,7 @@
         <v>7530</v>
       </c>
       <c r="M97" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16301,7 +16301,7 @@
         <v>5552</v>
       </c>
       <c r="M98" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16342,7 +16342,7 @@
         <v>5036</v>
       </c>
       <c r="M99" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16383,7 +16383,7 @@
         <v>1515</v>
       </c>
       <c r="M100" s="3" t="s">
-        <v>32</v>
+        <v>908</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>